<commit_message>
Update course plans for Italian and Spanish programs
- Revised learning outcomes for GIT3KP, GIT3KR, GSP3KS, GSP3KT, GSP3KU, GSP3KV, GTY3KJ, and GTY3KK to enhance clarity and correctness.
- Corrected spelling errors and improved language usage throughout course descriptions.
- Updated assessment methods and grading criteria for several courses to reflect current standards.
- Adjusted course content descriptions to better align with learning objectives and enhance student understanding.
- Modified scrape_hash values for all updated course plans.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/03 IKS/Analys/Övrigt.xlsx
+++ b/vault-dalarna-university/03 IKS/Analys/Övrigt.xlsx
@@ -2860,7 +2860,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Saknar standardfras om pedagogiskt stöd: Antal examinationsförsök är begränsat till fem. Den som antagits till och registrerats på kursen har rätt att erhålla un…</t>
+          <t>Saknar standardfras om pedagogiskt stöd: Antal examinationsförsök är begränsat till fem.…</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -2926,7 +2926,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Saknar standardfras om pedagogiskt stöd: Antal examinationsförsök är begränsat till fem. Den som antagits till och registrerats på kursen har rätt att erhålla un…</t>
+          <t>Saknar standardfras om pedagogiskt stöd: Antal examinationsförsök är begränsat till fem.…</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">

</xml_diff>